<commit_message>
Fix auto-save bug: skip empty/NaN rows in description lookup editor
Empty rows in data_editor caused '✓ Added nan' toast spam.
Now checks pd.isna() and filters string 'nan' before processing.

Co-authored-by: Qwen-Coder <qwen-coder@alibabacloud.com>
</commit_message>
<xml_diff>
--- a/Manifest Description Conversion.xlsx
+++ b/Manifest Description Conversion.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C341"/>
+  <dimension ref="A1:C342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6085,13 +6085,18 @@
       <c r="C340" t="inlineStr"/>
     </row>
     <row r="341">
-      <c r="A341" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="A341" t="inlineStr"/>
       <c r="B341" t="inlineStr"/>
       <c r="C341" t="inlineStr"/>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr"/>
+      <c r="C342" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>